<commit_message>
Update momentum code and allocation data for dashboard push
</commit_message>
<xml_diff>
--- a/Sectorwise_equity_allocation.xlsx
+++ b/Sectorwise_equity_allocation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anike\Desktop\Ocean_dev\Momentum Handover\Momentum Handover\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Ocean Finvest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AD1EA1C-6D4C-405C-81D9-069A8CE12C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03505F91-B9E4-402F-B2E7-017BEC353AD7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBDC62EB-6F6E-481F-A867-5258D773644F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15200" windowHeight="6810" xr2:uid="{EBDC62EB-6F6E-481F-A867-5258D773644F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>SECTOR</t>
   </si>
@@ -59,20 +48,23 @@
     <t>Metals &amp; Mining</t>
   </si>
   <si>
-    <t>Chemicals</t>
-  </si>
-  <si>
     <t>Power</t>
   </si>
   <si>
     <t>Percent_Allocation</t>
+  </si>
+  <si>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <t>Textiles</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,10 +109,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,84 +449,101 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA72E39E-FF48-4D45-98DF-AF69F66BC915}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.75" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B9" s="3">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B10" s="3">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2">
-        <v>0.05</v>
-      </c>
+      <c r="C10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>